<commit_message>
Add paragraph rephrasing: 50-example dataset, T5/Mac eval, LLM comparison Excel; update final_comparison.xlsx
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/final_comparison.xlsx
+++ b/final_comparison.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/chaks/Desktop/slm_edit/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DE90CD1-6ACB-EE45-BD2E-A105A5F57988}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3B1C91F-DAD0-5842-A455-3412DA029355}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5800" yWindow="3560" windowWidth="34560" windowHeight="20520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6540" yWindow="2220" windowWidth="34560" windowHeight="20500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Comparison_Table" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="30">
   <si>
     <t>Category</t>
   </si>
@@ -103,13 +103,22 @@
   </si>
   <si>
     <t>T5: model_evaluation_expanded_report.xlsx. Mac Typo/Grammar: mac_foundation_model_evaluation.xlsx. Mac Rephrasing: mac_rephrasing_only_results.xlsx.</t>
+  </si>
+  <si>
+    <t>Rephrasing (Sentence)</t>
+  </si>
+  <si>
+    <t>Rephrasing (Paragraph)</t>
+  </si>
+  <si>
+    <t>Test Set Size</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -122,9 +131,18 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -137,8 +155,20 @@
         <bgColor rgb="FF366092"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor rgb="FF366092"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor rgb="FF366092"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -161,14 +191,161 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -639,127 +816,147 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.1640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C1" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="15" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A2" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="2">
+        <v>100</v>
+      </c>
+      <c r="C2" s="2">
         <v>4.37</v>
       </c>
-      <c r="C2">
+      <c r="D2" s="9">
         <v>4.68</v>
       </c>
-      <c r="D2">
+      <c r="E2" s="2">
         <v>79</v>
       </c>
-      <c r="E2">
+      <c r="F2" s="9">
         <v>90</v>
       </c>
-      <c r="F2">
+      <c r="G2" s="2">
         <v>75</v>
       </c>
-      <c r="G2">
+      <c r="H2" s="12">
         <v>90</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="2">
+        <v>100</v>
+      </c>
+      <c r="C3" s="2">
         <v>3.25</v>
       </c>
-      <c r="C3">
+      <c r="D3" s="9">
         <v>4.1900000000000004</v>
       </c>
-      <c r="D3">
+      <c r="E3" s="2">
         <v>41</v>
       </c>
-      <c r="E3">
+      <c r="F3" s="9">
         <v>74</v>
       </c>
-      <c r="F3">
+      <c r="G3" s="2">
         <v>37</v>
       </c>
-      <c r="G3">
+      <c r="H3" s="12">
         <v>70</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>13</v>
-      </c>
-      <c r="B4">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A4" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" s="2">
+        <v>100</v>
+      </c>
+      <c r="C4" s="2">
         <v>1.28</v>
       </c>
-      <c r="C4">
+      <c r="D4" s="9">
         <v>4.08</v>
       </c>
-      <c r="D4">
+      <c r="E4" s="2">
         <v>2</v>
       </c>
-      <c r="E4">
+      <c r="F4" s="9">
         <v>80</v>
       </c>
-      <c r="F4">
+      <c r="G4" s="2">
         <v>2</v>
       </c>
-      <c r="G4">
+      <c r="H4" s="12">
         <v>41</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>14</v>
-      </c>
-      <c r="C5">
-        <v>4.3166666666666673</v>
-      </c>
-      <c r="D5">
-        <v>122</v>
-      </c>
-      <c r="E5">
-        <v>244</v>
-      </c>
-      <c r="F5">
-        <v>114</v>
-      </c>
-      <c r="G5">
-        <v>201</v>
+    <row r="5" spans="1:8" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" s="7">
+        <v>50</v>
+      </c>
+      <c r="C5" s="8">
+        <v>1.3</v>
+      </c>
+      <c r="D5" s="10">
+        <v>4.2</v>
+      </c>
+      <c r="E5" s="7">
+        <v>0</v>
+      </c>
+      <c r="F5" s="11">
+        <v>49</v>
+      </c>
+      <c r="G5" s="7">
+        <v>0</v>
+      </c>
+      <c r="H5" s="13">
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>